<commit_message>
nisip pentru constructii Adeplast: descriere SEO/GEO (intrebari frecvente, local) + fisa tehnica Rev.3 2023 gazduita pe site (link-ul Sika era mort)
</commit_message>
<xml_diff>
--- a/db/catalog/1-constructii_complet_MU.xlsx
+++ b/db/catalog/1-constructii_complet_MU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produse" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicționar tag-uri" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Produse" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dicționar tag-uri" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produse'!$A$1:$R$148</definedName>
@@ -6123,11 +6123,11 @@
       <c r="M47" s="3" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;strong&gt;Nisip ambalat pentru mortarele pe care le prepari singur&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;Nisipul pentru construcții Adeplast are granulație 0–1 mm și se livrează în sac de 25 kg, ușor de transportat și de depozitat. Este un agregat mineral spălat, sortat și fără argilă, conform SR EN 13139. Îl folosești împreună cu ciment și/sau var pentru mortare de tencuială, mortare de zidărie și șape.&lt;/p&gt;
+&lt;p&gt;Nisipul pentru construcții Adeplast are granulație 0–1 mm și se livrează în sac de 25 kg, ușor de transportat și de depozitat. Este un agregat mineral spălat, sortat și fără argilă, conform SR EN 13139. Îl amesteci cu ciment și/sau var ca să obții mortar de tencuială, mortar de zidărie, tinci sau șapă de egalizare, direct pe șantier.&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Calitate constantă&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;Granulația controlată și lipsa argilei îți dau mortare omogene, cu aceeași consistență la fiecare amestec.&lt;/p&gt;
+&lt;p&gt;Granulația controlată și lipsa argilei îți dau mortare omogene, cu aceeași consistență la fiecare amestec — fără pietre, fără bulgări și fără să-l mai cerni.&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Dozare ușoară&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;Pentru că sacul are o greutate fixă, poți urmări direct proporțiile de ciment recomandate de producător.&lt;/p&gt;
+&lt;p&gt;Sacul are o greutate fixă, deci urmărești direct proporțiile de ciment recomandate de producător, fără să cântărești nisipul.&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Proporții recomandate (25 kg nisip uscat)&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
 &lt;li&gt;Mortar de zidărie: 5 kg ciment.&lt;/li&gt;
@@ -6137,7 +6137,12 @@
 &lt;li&gt;Lucrează la temperaturi ale aerului și suportului între +5 și +30 °C; peste +25 °C umezește suplimentar suprafața, ca să eviți fisurarea.&lt;/li&gt;
 &lt;/ul&gt;
 &lt;p&gt;&lt;strong&gt;Limitări&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;Mortarele preparate cu acest nisip nu se recomandă pe lemn, materiale plastice, metale sau suprafețe din ipsos. Evită bătaia directă a soarelui și protejează suprafețele de uscarea rapidă, intemperii și îngheț. Nisipul poate conține urme de ciment din procesul de fabricație. Sacul se păstrează 12 luni de la fabricație, în spațiu uscat, pe paleți de lemn.&lt;/p&gt;</t>
+&lt;p&gt;Mortarele preparate cu acest nisip nu se recomandă pe lemn, materiale plastice, metale sau suprafețe din ipsos. Evită bătaia directă a soarelui și protejează suprafețele de uscarea rapidă, intemperii și îngheț. Nisipul poate conține urme de ciment din procesul de fabricație. Sacul se păstrează 12 luni de la fabricație, în spațiu uscat, pe paleți de lemn.&lt;/p&gt;
+&lt;h3&gt;Întrebări frecvente&lt;/h3&gt;
+&lt;p&gt;&lt;strong&gt;Cât ciment pun la un sac de nisip de 25 kg?&lt;/strong&gt;&lt;br&gt;Depinde de lucrare: 5 kg ciment pentru mortar de zidărie sau de tencuială, 6 kg pentru tinci și 7 kg pentru șapă de egalizare, conform fișei tehnice Adeplast.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Prin ce diferă de nisipul cuarțos Adeplast?&lt;/strong&gt;&lt;br&gt;Ambele au granulație 0–1 mm și aceleași proporții de ciment. Nisipul cuarțos este recomandat în plus pentru înglobarea în pardoselile din rășini epoxidice; pentru tencuieli, zidărie și șape obișnuite, nisipul pentru construcții este suficient.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Îl pot folosi pe gips-carton, lemn sau metal?&lt;/strong&gt;&lt;br&gt;Nu. Producătorul nu recomandă mortarele făcute cu acest nisip pe lemn, plastic, metal sau ipsos — pentru gips-carton alege un glet sau un adeziv dedicat.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;De unde îl iau în zona Dăbuleni?&lt;/strong&gt;&lt;br&gt;Îl găsești la magazinul Mugurel din Dăbuleni (Strada Caracal 66), în saci de 25 kg. Poți comanda online sau pe WhatsApp: te sunăm să confirmăm stocul, iar livrarea se face în județul Dolj.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr">
@@ -6157,11 +6162,7 @@
 Nu se aplică pe: lemn, materiale plastice, metale, suprafețe din ipsos</t>
         </is>
       </c>
-      <c r="O47" s="3" t="inlineStr">
-        <is>
-          <t>https://rou.sika.com/dms/getdocument.get/5d31b836-2e7b-4f71-b693-95a8da3cad43_ro01/nisip-pentru-constructii0-1mm.pdf</t>
-        </is>
-      </c>
+      <c r="O47" s="3" t="n"/>
       <c r="P47" s="3" t="inlineStr">
         <is>
           <t>https://rou.sika.com/ro/adeplast/adeplast-mortare-uscate/adeplast-mortare-de-tencuiala/nisip-pentru-constructii.html | https://www.hornbach.ro/p/nisip-adeplast-pentru-constructii-granulatie-0-1-1-mm-25-kg/8576693/ | https://media.hornbach.ro/hb/technicaldatasheet/as.144226735.pdf</t>
@@ -6174,7 +6175,7 @@
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t>Cod de bare confirmat pe Hornbach. Fișa de pe site-ul Sika este Ed.3 din 11.05.2020; pe Hornbach există o revizie mai nouă (Rev.3, 02.10.2023), cu aceleași date plus standardul SR EN 13139 și mențiunea despre urmele de ciment, pe care le-am preluat. Hornbach scrie granulație 0,1–1 mm în titlu; ambele fișe scriu 0–1 mm (am folosit fișa). Densitatea (1.500 kg/m³) și culoarea bej apar doar pe Hornbach, așa că nu le-am preluat. Atenție: fișa tehnică e practic identică cu cea a nisipului cuarțos Adeplast (alt cod de bare, alt produs în ERP).</t>
+          <t>Cod de bare confirmat pe Hornbach. Fișa de pe site-ul Sika este Ed.3 din 11.05.2020; pe Hornbach există o revizie mai nouă (Rev.3, 02.10.2023), cu aceleași date plus standardul SR EN 13139 și mențiunea despre urmele de ciment, pe care le-am preluat. Hornbach scrie granulație 0,1–1 mm în titlu; ambele fișe scriu 0–1 mm (am folosit fișa). Densitatea (1.500 kg/m³) și culoarea bej apar doar pe Hornbach, așa că nu le-am preluat. Atenție: fișa tehnică e practic identică cu cea a nisipului cuarțos Adeplast (alt cod de bare, alt produs în ERP). | 17 oct 2026: descriere extinsa (intrebari frecvente, local); fisa tehnica Rev.3 2023 gazduita pe site (fise-tehnice/), link-ul Sika dadea 404.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update 2: tema intunecata (manuala), electrocasnice varianta 2 cu descrieri complete, fise moarte scoase
- tema intunecata doar din butonul soare/luna; implicit luminoasa; aplicata inainte de afisare (fara clipire);
  culorile CSS trecute pe variabile, tema luminoasa ramasa identica (comparatie de capturi); contrast verificat
- electrocasnice: fisierul „varianta 2" (aceleasi produse si preturi); toate 200 au acum descriere si specificatii
  (26 completate din surse verificate, valorile contradictorii lasate deoparte)
- fise tehnice: linkurile moarte (404) scoase; linkurile EPREL afisate ca „Eticheta energetica", nu „PDF"
</commit_message>
<xml_diff>
--- a/db/catalog/1-constructii_complet_MU.xlsx
+++ b/db/catalog/1-constructii_complet_MU.xlsx
@@ -2224,11 +2224,7 @@
 Nu se aplică pe: lemn, plastic, metal</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>https://rou.sika.com/dms/getdocument.get/cc35eba1-de73-4792-b72c-21fba6473e73_ro01/adeziv-pentru-placitermoizolantepolistiren.pdf</t>
-        </is>
-      </c>
+      <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="inlineStr">
         <is>
           <t>https://rou.sika.com/ro/adeplast/adeplast-mortare-uscate/adeplast-adezivi-pentru-termoizolatii/polistirol-eco-plus.html | https://www.evoracenter.ro/adeziv-polistirol-eco-plus-25kg</t>
@@ -2241,7 +2237,7 @@
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>Denumirea din ERP („Polistirol Plus”) nu corespunde: codul de bare (confirmat pe evoracenter.ro) este al produsului Polistirol Eco Plus; recomand corectarea în ERP. Culoarea nu apare în nicio sursă, deci am omis-o. Fișa dă apa în l/kg; n-am recalculat-o pe sac.</t>
+          <t>Denumirea din ERP („Polistirol Plus”) nu corespunde: codul de bare (confirmat pe evoracenter.ro) este al produsului Polistirol Eco Plus; recomand corectarea în ERP. Culoarea nu apare în nicio sursă, deci am omis-o. Fișa dă apa în l/kg; n-am recalculat-o pe sac. | 18 oct 2026: link de fișă scos (404 la producător, fără înlocuitor oficial).</t>
         </is>
       </c>
     </row>
@@ -5919,11 +5915,7 @@
 Termen de valabilitate: 12 luni de la data fabricației</t>
         </is>
       </c>
-      <c r="O45" s="3" t="inlineStr">
-        <is>
-          <t>https://rou.sika.com/content/dam/dms/ro01/f/mortar-de-zidariemz5pentruconstructii.pdf</t>
-        </is>
-      </c>
+      <c r="O45" s="3" t="n"/>
       <c r="P45" s="3" t="inlineStr">
         <is>
           <t>https://rou.sika.com/ro/adeplast/adeplast-mortare-uscate/adeplast-mortare-pentru-zidarie/mz-5.html | https://amset.ro/wp-content/uploads/2025/07/540-Fisa-tehnica-ADEPLAST-MZ-5-2018.pdf | https://www.evoracenter.ro/?id=1448&amp;pid=1769102 | https://www.leroymerlin.ro/produse/mortar-zidarie-adeplast-mz-5-interior-exterior-30-kg-11467750.html</t>
@@ -5936,7 +5928,7 @@
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t>Cod de bare confirmat pe evoracenter.ro („MORTAR ZIDARIE MZ-50 30KG”, unde apare ca ieșit din ofertă). Pe site-ul Sika produsul se numește „MZ - 5”; „MZ-50” e denumirea din ERP și de la unii retaileri. Fișa oficială Sika nu s-a putut deschide; datele sunt din fișa tehnică Adeplast DP-61 Ed.2 din 04.12.2018 (copie pe amset.ro), de verificat dacă există o ediție mai nouă. Regata.ro indică 5,4–6,0 l apă la sac; am folosit fișa (4,2–5,4 l). Culoarea gri e confirmată doar de Leroy Merlin (fișa nu o precizează). Fișa spune „destinat în construcții exterioare”, Leroy Merlin „interior/exterior”; n-am trecut locul de utilizare în denumire/tag-uri.</t>
+          <t>Cod de bare confirmat pe evoracenter.ro („MORTAR ZIDARIE MZ-50 30KG”, unde apare ca ieșit din ofertă). Pe site-ul Sika produsul se numește „MZ - 5”; „MZ-50” e denumirea din ERP și de la unii retaileri. Fișa oficială Sika nu s-a putut deschide; datele sunt din fișa tehnică Adeplast DP-61 Ed.2 din 04.12.2018 (copie pe amset.ro), de verificat dacă există o ediție mai nouă. Regata.ro indică 5,4–6,0 l apă la sac; am folosit fișa (4,2–5,4 l). Culoarea gri e confirmată doar de Leroy Merlin (fișa nu o precizează). Fișa spune „destinat în construcții exterioare”, Leroy Merlin „interior/exterior”; n-am trecut locul de utilizare în denumire/tag-uri. | 18 oct 2026: link de fișă scos (404 la producător, fără înlocuitor oficial).</t>
         </is>
       </c>
     </row>

</xml_diff>